<commit_message>
fix: add Android SDK setup to GHA pipeline and resolve API load test timeouts
</commit_message>
<xml_diff>
--- a/PythonTesting/reports/Automation_Test_Report.xlsx
+++ b/PythonTesting/reports/Automation_Test_Report.xlsx
@@ -46673,7 +46673,7 @@
       </c>
       <c r="F1642" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1555ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1947ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -47321,7 +47321,7 @@
       </c>
       <c r="F1665" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1933ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1688ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -47969,7 +47969,7 @@
       </c>
       <c r="F1688" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1645ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1790ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -48617,7 +48617,7 @@
       </c>
       <c r="F1711" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1739ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1756ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -49265,7 +49265,7 @@
       </c>
       <c r="F1734" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1794ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1939ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -49913,7 +49913,7 @@
       </c>
       <c r="F1757" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1713ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1706ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -50561,7 +50561,7 @@
       </c>
       <c r="F1780" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1922ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1784ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -51209,7 +51209,7 @@
       </c>
       <c r="F1803" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1631ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1621ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -51857,7 +51857,7 @@
       </c>
       <c r="F1826" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1766ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1874ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -52505,7 +52505,7 @@
       </c>
       <c r="F1849" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1725ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1901ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -53153,7 +53153,7 @@
       </c>
       <c r="F1872" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1944ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1785ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -53801,7 +53801,7 @@
       </c>
       <c r="F1895" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1705ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1933ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -54449,7 +54449,7 @@
       </c>
       <c r="F1918" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1669ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1749ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -55097,7 +55097,7 @@
       </c>
       <c r="F1941" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1803ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1667ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -55745,7 +55745,7 @@
       </c>
       <c r="F1964" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1789ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1821ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -56393,7 +56393,7 @@
       </c>
       <c r="F1987" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1561ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1859ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -57041,7 +57041,7 @@
       </c>
       <c r="F2010" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1586ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1939ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement parallel multi-job GHA pipeline graph and report bundling
</commit_message>
<xml_diff>
--- a/PythonTesting/reports/Automation_Test_Report.xlsx
+++ b/PythonTesting/reports/Automation_Test_Report.xlsx
@@ -46673,7 +46673,7 @@
       </c>
       <c r="F1642" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1947ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1705ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -47321,7 +47321,7 @@
       </c>
       <c r="F1665" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1688ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1934ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -47969,7 +47969,7 @@
       </c>
       <c r="F1688" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1790ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1879ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -48617,7 +48617,7 @@
       </c>
       <c r="F1711" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1756ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1777ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -49265,7 +49265,7 @@
       </c>
       <c r="F1734" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1939ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1782ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -49913,7 +49913,7 @@
       </c>
       <c r="F1757" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1706ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1707ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -50561,7 +50561,7 @@
       </c>
       <c r="F1780" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1784ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1743ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -51209,7 +51209,7 @@
       </c>
       <c r="F1803" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1621ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1861ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -51857,7 +51857,7 @@
       </c>
       <c r="F1826" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1874ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1773ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -52505,7 +52505,7 @@
       </c>
       <c r="F1849" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1901ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1890ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -53153,7 +53153,7 @@
       </c>
       <c r="F1872" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1785ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1686ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -53801,7 +53801,7 @@
       </c>
       <c r="F1895" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1933ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1582ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -54449,7 +54449,7 @@
       </c>
       <c r="F1918" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1749ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1712ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -55097,7 +55097,7 @@
       </c>
       <c r="F1941" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1667ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1928ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -55745,7 +55745,7 @@
       </c>
       <c r="F1964" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1821ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1902ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -56393,7 +56393,7 @@
       </c>
       <c r="F1987" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1859ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1835ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>
@@ -57041,7 +57041,7 @@
       </c>
       <c r="F2010" s="2" t="inlineStr">
         <is>
-          <t>Latency SLA Violation: P95 Response latency of 1939ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
+          <t>Latency SLA Violation: P95 Response latency of 1783ms exceeded target threshold of 1500ms under 100 VU concurrent load.</t>
         </is>
       </c>
     </row>

</xml_diff>